<commit_message>
Add Jam drawing to visualize
</commit_message>
<xml_diff>
--- a/globallbz1_p_ttl_10.xlsx
+++ b/globallbz1_p_ttl_10.xlsx
@@ -675,10 +675,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B2" t="n">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C2" t="n">
         <v>30000</v>
@@ -687,38 +687,44 @@
         <v>5052</v>
       </c>
       <c r="E2" t="n">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="F2" t="n">
-        <v>235</v>
+        <v>202</v>
       </c>
       <c r="G2" t="n">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="H2" t="n">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="I2" t="n">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="J2" t="n">
-        <v>244</v>
+        <v>113</v>
       </c>
       <c r="K2" t="n">
-        <v>1416.206542346071</v>
+        <v>1424.11333620486</v>
       </c>
       <c r="L2" t="n">
         <v>8</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>289</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1749.514762748161</v>
+      </c>
+      <c r="O2" t="n">
+        <v>8</v>
+      </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>171.5453638279912</t>
+          <t>167.9523929280221</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -727,40 +733,40 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B3" t="n">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="C3" t="n">
         <v>30000</v>
       </c>
       <c r="D3" t="n">
-        <v>5056</v>
+        <v>5052</v>
       </c>
       <c r="E3" t="n">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="F3" t="n">
-        <v>234.75</v>
+        <v>194.5</v>
       </c>
       <c r="G3" t="n">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="H3" t="n">
-        <v>127</v>
+        <v>139.5</v>
       </c>
       <c r="I3" t="n">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="J3" t="n">
-        <v>245</v>
+        <v>195</v>
       </c>
       <c r="K3" t="n">
-        <v>1591.578626228542</v>
+        <v>1479.867509086479</v>
       </c>
       <c r="L3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -770,7 +776,7 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>168.1877157650203</t>
+          <t>163.9857348261569</t>
         </is>
       </c>
       <c r="T3" t="n">
@@ -779,10 +785,10 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="B4" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="C4" t="n">
         <v>30000</v>
@@ -791,25 +797,25 @@
         <v>5056</v>
       </c>
       <c r="E4" t="n">
+        <v>120</v>
+      </c>
+      <c r="F4" t="n">
+        <v>234</v>
+      </c>
+      <c r="G4" t="n">
         <v>123</v>
       </c>
-      <c r="F4" t="n">
-        <v>177.9166666666667</v>
-      </c>
-      <c r="G4" t="n">
-        <v>126</v>
-      </c>
       <c r="H4" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I4" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="J4" t="n">
-        <v>213</v>
+        <v>234</v>
       </c>
       <c r="K4" t="n">
-        <v>1556.2860407945</v>
+        <v>1564.068492725869</v>
       </c>
       <c r="L4" t="n">
         <v>9</v>
@@ -822,7 +828,7 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>173.86227100766843</t>
+          <t>165.79020175607732</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -831,10 +837,10 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B5" t="n">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="C5" t="n">
         <v>30000</v>
@@ -843,25 +849,25 @@
         <v>5056</v>
       </c>
       <c r="E5" t="n">
-        <v>142</v>
+        <v>183</v>
       </c>
       <c r="F5" t="n">
-        <v>176.8</v>
+        <v>223.5714285714286</v>
       </c>
       <c r="G5" t="n">
-        <v>142</v>
+        <v>183</v>
       </c>
       <c r="H5" t="n">
-        <v>145</v>
+        <v>189.6666666666667</v>
       </c>
       <c r="I5" t="n">
-        <v>142</v>
+        <v>183</v>
       </c>
       <c r="J5" t="n">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="K5" t="n">
-        <v>1562.786033474744</v>
+        <v>1703.93803932479</v>
       </c>
       <c r="L5" t="n">
         <v>9</v>
@@ -874,7 +880,7 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>168.0104616717245</t>
+          <t>168.2279390907692</t>
         </is>
       </c>
       <c r="T5" t="n">
@@ -883,10 +889,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="B6" t="n">
-        <v>91</v>
+        <v>142</v>
       </c>
       <c r="C6" t="n">
         <v>30000</v>
@@ -895,25 +901,25 @@
         <v>5056</v>
       </c>
       <c r="E6" t="n">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="F6" t="n">
-        <v>141.3333333333333</v>
+        <v>168.7142857142857</v>
       </c>
       <c r="G6" t="n">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="H6" t="n">
-        <v>141.3333333333333</v>
+        <v>120</v>
       </c>
       <c r="I6" t="n">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="J6" t="n">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="K6" t="n">
-        <v>1668.731540647929</v>
+        <v>1563.402914689668</v>
       </c>
       <c r="L6" t="n">
         <v>9</v>
@@ -926,7 +932,7 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>168.81118190359805</t>
+          <t>166.25597972246788</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -935,40 +941,40 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B7" t="n">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="C7" t="n">
         <v>30000</v>
       </c>
       <c r="D7" t="n">
-        <v>5060</v>
+        <v>5056</v>
       </c>
       <c r="E7" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F7" t="n">
-        <v>168.8</v>
+        <v>182.3636363636364</v>
       </c>
       <c r="G7" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H7" t="n">
-        <v>139</v>
+        <v>130.5</v>
       </c>
       <c r="I7" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J7" t="n">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="K7" t="n">
-        <v>1846.562458754093</v>
+        <v>1631.554620291809</v>
       </c>
       <c r="L7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -978,7 +984,7 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>168.5794448850079</t>
+          <t>166.15366820817312</t>
         </is>
       </c>
       <c r="T7" t="n">
@@ -987,40 +993,40 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B8" t="n">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="C8" t="n">
         <v>30000</v>
       </c>
       <c r="D8" t="n">
-        <v>5056</v>
+        <v>5052</v>
       </c>
       <c r="E8" t="n">
-        <v>129</v>
+        <v>205</v>
       </c>
       <c r="F8" t="n">
-        <v>205.6666666666667</v>
+        <v>214</v>
       </c>
       <c r="G8" t="n">
-        <v>129</v>
+        <v>234</v>
       </c>
       <c r="H8" t="n">
-        <v>134.7857142857143</v>
+        <v>214</v>
       </c>
       <c r="I8" t="n">
-        <v>129</v>
+        <v>205</v>
       </c>
       <c r="J8" t="n">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="K8" t="n">
-        <v>1495.978962995963</v>
+        <v>1290.31441436713</v>
       </c>
       <c r="L8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
@@ -1030,7 +1036,7 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>164.81289404905172</t>
+          <t>165.83954133545595</t>
         </is>
       </c>
       <c r="T8" t="n">
@@ -1039,10 +1045,10 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B9" t="n">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="C9" t="n">
         <v>30000</v>
@@ -1051,25 +1057,25 @@
         <v>5056</v>
       </c>
       <c r="E9" t="n">
-        <v>155</v>
+        <v>209</v>
       </c>
       <c r="F9" t="n">
-        <v>177.6666666666667</v>
+        <v>221.8</v>
       </c>
       <c r="G9" t="n">
-        <v>155</v>
+        <v>218</v>
       </c>
       <c r="H9" t="n">
-        <v>169</v>
+        <v>213.6666666666667</v>
       </c>
       <c r="I9" t="n">
-        <v>155</v>
+        <v>209</v>
       </c>
       <c r="J9" t="n">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="K9" t="n">
-        <v>1534.837053883674</v>
+        <v>1447.043031079404</v>
       </c>
       <c r="L9" t="n">
         <v>9</v>
@@ -1082,7 +1088,7 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>171.7524100796294</t>
+          <t>160.8718328444182</t>
         </is>
       </c>
       <c r="T9" t="n">
@@ -1091,7 +1097,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B10" t="n">
         <v>81</v>
@@ -1100,41 +1106,47 @@
         <v>30000</v>
       </c>
       <c r="D10" t="n">
-        <v>5056</v>
+        <v>5052</v>
       </c>
       <c r="E10" t="n">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="F10" t="n">
-        <v>170.3333333333333</v>
+        <v>155.1052631578947</v>
       </c>
       <c r="G10" t="n">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="H10" t="n">
-        <v>170.3333333333333</v>
+        <v>129.5</v>
       </c>
       <c r="I10" t="n">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="J10" t="n">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="K10" t="n">
-        <v>1434.808685612507</v>
+        <v>1442.356725184032</v>
       </c>
       <c r="L10" t="n">
-        <v>9</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="M10" t="n">
+        <v>188</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1384.100390051574</v>
+      </c>
+      <c r="O10" t="n">
+        <v>8</v>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>160.03196063918867</t>
+          <t>176.05647776490287</t>
         </is>
       </c>
       <c r="T10" t="n">
@@ -1143,62 +1155,40 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B11" t="n">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="C11" t="n">
         <v>30000</v>
       </c>
       <c r="D11" t="n">
-        <v>5056</v>
-      </c>
-      <c r="E11" t="n">
-        <v>122</v>
-      </c>
-      <c r="F11" t="n">
-        <v>201.75</v>
-      </c>
-      <c r="G11" t="n">
-        <v>122</v>
-      </c>
-      <c r="H11" t="n">
-        <v>123.2</v>
-      </c>
-      <c r="I11" t="n">
-        <v>122</v>
-      </c>
-      <c r="J11" t="n">
-        <v>217</v>
-      </c>
-      <c r="K11" t="n">
-        <v>1664.808886593527</v>
-      </c>
-      <c r="L11" t="n">
-        <v>9</v>
-      </c>
+        <v>5064</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>170.8001698685842</t>
-        </is>
-      </c>
-      <c r="T11" t="n">
-        <v>10</v>
-      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B12" t="n">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="C12" t="n">
         <v>30000</v>
@@ -1207,25 +1197,25 @@
         <v>5056</v>
       </c>
       <c r="E12" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F12" t="n">
-        <v>153.03125</v>
+        <v>149.8</v>
       </c>
       <c r="G12" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="H12" t="n">
-        <v>111.5</v>
+        <v>115.25</v>
       </c>
       <c r="I12" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="J12" t="n">
-        <v>153</v>
+        <v>111</v>
       </c>
       <c r="K12" t="n">
-        <v>1737.715902816122</v>
+        <v>1689.580671765478</v>
       </c>
       <c r="L12" t="n">
         <v>9</v>
@@ -1238,7 +1228,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>169.91732269944873</t>
+          <t>170.0991715002953</t>
         </is>
       </c>
       <c r="T12" t="n">
@@ -1247,40 +1237,40 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C13" t="n">
         <v>30000</v>
       </c>
       <c r="D13" t="n">
-        <v>5052</v>
+        <v>5056</v>
       </c>
       <c r="E13" t="n">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="F13" t="n">
-        <v>223</v>
+        <v>159.40625</v>
       </c>
       <c r="G13" t="n">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="H13" t="n">
-        <v>149.5</v>
+        <v>130</v>
       </c>
       <c r="I13" t="n">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="J13" t="n">
-        <v>223</v>
+        <v>173</v>
       </c>
       <c r="K13" t="n">
-        <v>1383.555956921019</v>
+        <v>1649.882581995727</v>
       </c>
       <c r="L13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1290,7 +1280,7 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>164.32618469965473</t>
+          <t>159.5348685840656</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -1299,40 +1289,40 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B14" t="n">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="C14" t="n">
         <v>30000</v>
       </c>
       <c r="D14" t="n">
-        <v>5056</v>
+        <v>5060</v>
       </c>
       <c r="E14" t="n">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="F14" t="n">
-        <v>146.2222222222222</v>
+        <v>164.4615384615385</v>
       </c>
       <c r="G14" t="n">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="H14" t="n">
-        <v>116</v>
+        <v>128.5</v>
       </c>
       <c r="I14" t="n">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="J14" t="n">
-        <v>211</v>
+        <v>126</v>
       </c>
       <c r="K14" t="n">
-        <v>1594.536683554159</v>
+        <v>1749.172745701303</v>
       </c>
       <c r="L14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
@@ -1342,7 +1332,7 @@
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>166.8327073544929</t>
+          <t>174.92821896826257</t>
         </is>
       </c>
       <c r="T14" t="n">
@@ -1351,40 +1341,40 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="B15" t="n">
-        <v>112</v>
+        <v>149</v>
       </c>
       <c r="C15" t="n">
         <v>30000</v>
       </c>
       <c r="D15" t="n">
-        <v>5056</v>
+        <v>5052</v>
       </c>
       <c r="E15" t="n">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="F15" t="n">
-        <v>231.3333333333333</v>
+        <v>184</v>
       </c>
       <c r="G15" t="n">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="H15" t="n">
         <v>159</v>
       </c>
       <c r="I15" t="n">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="J15" t="n">
-        <v>262</v>
+        <v>159</v>
       </c>
       <c r="K15" t="n">
-        <v>1346.502507348086</v>
+        <v>1603.212763787735</v>
       </c>
       <c r="L15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
@@ -1394,7 +1384,7 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>164.02430931664983</t>
+          <t>171.92514829045572</t>
         </is>
       </c>
       <c r="T15" t="n">
@@ -1403,10 +1393,10 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B16" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C16" t="n">
         <v>30000</v>
@@ -1415,25 +1405,25 @@
         <v>5056</v>
       </c>
       <c r="E16" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F16" t="n">
-        <v>225.3333333333333</v>
+        <v>249.3333333333333</v>
       </c>
       <c r="G16" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H16" t="n">
-        <v>123.3333333333333</v>
+        <v>115</v>
       </c>
       <c r="I16" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J16" t="n">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="K16" t="n">
-        <v>1650.896083070469</v>
+        <v>1610.628064579817</v>
       </c>
       <c r="L16" t="n">
         <v>9</v>
@@ -1446,7 +1436,7 @@
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>167.2461878425074</t>
+          <t>172.87092646898435</t>
         </is>
       </c>
       <c r="T16" t="n">
@@ -1455,56 +1445,50 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B17" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C17" t="n">
         <v>30000</v>
       </c>
       <c r="D17" t="n">
-        <v>5052</v>
+        <v>5060</v>
       </c>
       <c r="E17" t="n">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F17" t="n">
-        <v>226.25</v>
+        <v>148.0714285714286</v>
       </c>
       <c r="G17" t="n">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="H17" t="n">
-        <v>113</v>
+        <v>124.1666666666667</v>
       </c>
       <c r="I17" t="n">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="J17" t="n">
-        <v>212</v>
+        <v>161</v>
       </c>
       <c r="K17" t="n">
-        <v>1455.761177970195</v>
+        <v>1716.343223095213</v>
       </c>
       <c r="L17" t="n">
-        <v>8</v>
-      </c>
-      <c r="M17" t="n">
-        <v>286</v>
-      </c>
-      <c r="N17" t="n">
-        <v>1724.447438912231</v>
-      </c>
-      <c r="O17" t="n">
-        <v>8</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>162.84386443229494</t>
+          <t>163.623545131714</t>
         </is>
       </c>
       <c r="T17" t="n">
@@ -1513,40 +1497,40 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="B18" t="n">
-        <v>154</v>
+        <v>78</v>
       </c>
       <c r="C18" t="n">
         <v>30000</v>
       </c>
       <c r="D18" t="n">
-        <v>5056</v>
+        <v>5052</v>
       </c>
       <c r="E18" t="n">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="F18" t="n">
-        <v>213.64</v>
+        <v>222.5</v>
       </c>
       <c r="G18" t="n">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="H18" t="n">
-        <v>141.1666666666667</v>
+        <v>123.5</v>
       </c>
       <c r="I18" t="n">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="J18" t="n">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="K18" t="n">
-        <v>1664.603906001007</v>
+        <v>1504.683931165174</v>
       </c>
       <c r="L18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
@@ -1556,7 +1540,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>165.66492819107478</t>
+          <t>162.07891726118976</t>
         </is>
       </c>
       <c r="T18" t="n">
@@ -1565,40 +1549,40 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B19" t="n">
-        <v>83</v>
+        <v>121</v>
       </c>
       <c r="C19" t="n">
         <v>30000</v>
       </c>
       <c r="D19" t="n">
-        <v>5052</v>
+        <v>5056</v>
       </c>
       <c r="E19" t="n">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="F19" t="n">
-        <v>144</v>
+        <v>218</v>
       </c>
       <c r="G19" t="n">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="H19" t="n">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="I19" t="n">
-        <v>141</v>
+        <v>115</v>
       </c>
       <c r="J19" t="n">
-        <v>147</v>
+        <v>220</v>
       </c>
       <c r="K19" t="n">
-        <v>1563.615510895055</v>
+        <v>1545.294574102699</v>
       </c>
       <c r="L19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
@@ -1608,7 +1592,7 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>169.72543814250696</t>
+          <t>171.03023449496914</t>
         </is>
       </c>
       <c r="T19" t="n">
@@ -1617,40 +1601,40 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B20" t="n">
-        <v>133</v>
+        <v>83</v>
       </c>
       <c r="C20" t="n">
         <v>30000</v>
       </c>
       <c r="D20" t="n">
-        <v>5060</v>
+        <v>5056</v>
       </c>
       <c r="E20" t="n">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="F20" t="n">
-        <v>226.85</v>
+        <v>174.4761904761905</v>
       </c>
       <c r="G20" t="n">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="H20" t="n">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="I20" t="n">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="J20" t="n">
-        <v>214</v>
+        <v>147</v>
       </c>
       <c r="K20" t="n">
-        <v>1935.720304190436</v>
+        <v>1630.707269399363</v>
       </c>
       <c r="L20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
@@ -1660,7 +1644,7 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>164.73082836364054</t>
+          <t>157.9471506692625</t>
         </is>
       </c>
       <c r="T20" t="n">
@@ -1669,40 +1653,40 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B21" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="C21" t="n">
         <v>30000</v>
       </c>
       <c r="D21" t="n">
-        <v>5060</v>
+        <v>5056</v>
       </c>
       <c r="E21" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F21" t="n">
-        <v>205.7222222222222</v>
+        <v>210.1</v>
       </c>
       <c r="G21" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="H21" t="n">
-        <v>114.9411764705882</v>
+        <v>109.25</v>
       </c>
       <c r="I21" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="J21" t="n">
-        <v>234</v>
+        <v>187</v>
       </c>
       <c r="K21" t="n">
-        <v>1575.761199799247</v>
+        <v>1506.965096575111</v>
       </c>
       <c r="L21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
@@ -1712,7 +1696,7 @@
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>162.90179875321397</t>
+          <t>166.79943078281187</t>
         </is>
       </c>
       <c r="T21" t="n">

</xml_diff>